<commit_message>
new changes add to allur report result
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\STZ\eclipse-workspace\SwagLabProj_new\TestData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\STZ\eclipse-workspace\Swag-Lab-Project\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92C1C909-06D9-41BB-8608-4D455DF5D3B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27E68B3A-4F34-4D39-9821-4F3D1CF0255E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="22">
   <si>
     <t>standard_user</t>
   </si>
@@ -92,6 +92,15 @@
   </si>
   <si>
     <t>Sauce Labs Backpack</t>
+  </si>
+  <si>
+    <t>Third Item Purchase</t>
+  </si>
+  <si>
+    <t>Item to be removed</t>
+  </si>
+  <si>
+    <t>Remove Item</t>
   </si>
 </sst>
 </file>
@@ -187,7 +196,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -214,6 +223,7 @@
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -559,7 +569,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5547A6D9-B35F-4592-972E-BF4A3E31F7BE}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="31.88671875" customWidth="1"/>
@@ -613,7 +623,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="B4" s="7" t="s">
         <v>11</v>
@@ -623,6 +633,20 @@
       </c>
       <c r="D4" s="10">
         <v>7.99</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="10">
+        <v>15.99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>